<commit_message>
refactor(daq): stabilise pipeline and query sync
</commit_message>
<xml_diff>
--- a/src_matlab/stream_test/WindTunnel_Master_Result.xlsx
+++ b/src_matlab/stream_test/WindTunnel_Master_Result.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="17" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="37" uniqueCount="15">
   <si>
     <t>RunID</t>
   </si>
@@ -44,6 +44,21 @@
   </si>
   <si>
     <t>run_20260615_123476</t>
+  </si>
+  <si>
+    <t>run_20260615_124315</t>
+  </si>
+  <si>
+    <t>run_20260615_131120</t>
+  </si>
+  <si>
+    <t>drag</t>
+  </si>
+  <si>
+    <t>dyn_pressure</t>
+  </si>
+  <si>
+    <t>temperature</t>
   </si>
 </sst>
 </file>
@@ -89,14 +104,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20.140625" customWidth="true"/>
-    <col min="2" max="2" width="7.85546875" customWidth="true"/>
+    <col min="2" max="2" width="9.5703125" customWidth="true"/>
     <col min="3" max="3" width="11.7109375" customWidth="true"/>
     <col min="4" max="4" width="11.7109375" customWidth="true"/>
-    <col min="5" max="5" width="11.7109375" customWidth="true"/>
+    <col min="5" max="5" width="12.7109375" customWidth="true"/>
+    <col min="6" max="6" width="13.7109375" customWidth="true"/>
+    <col min="7" max="7" width="13.140625" customWidth="true"/>
+    <col min="8" max="8" width="12.42578125" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -115,56 +133,92 @@
       <c r="E1" s="0" t="s">
         <v>8</v>
       </c>
+      <c r="F1" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="G1" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="H1" s="0" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="B2" s="0" t="s">
         <v>3</v>
       </c>
       <c r="C2" s="0">
-        <v>49.174104248736541</v>
+        <v>30.02846622467041</v>
       </c>
       <c r="D2" s="0">
-        <v>3.9469891620445612</v>
+        <v>1.9992342591285706</v>
       </c>
       <c r="E2" s="0">
-        <v>16.041104391245295</v>
+        <v>0.50472483038902283</v>
+      </c>
+      <c r="F2" s="0">
+        <v>0.050472483038902283</v>
+      </c>
+      <c r="G2" s="0">
+        <v>552.29808044433594</v>
+      </c>
+      <c r="H2" s="0">
+        <v>24.974925994873047</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="B3" s="0" t="s">
         <v>4</v>
       </c>
       <c r="C3" s="0">
-        <v>49.025553051361257</v>
+        <v>49.937663078308105</v>
       </c>
       <c r="D3" s="0">
-        <v>4.0106468993167193</v>
+        <v>3.9882382154464722</v>
       </c>
       <c r="E3" s="0">
-        <v>16.076181834700417</v>
+        <v>1.2046135663986206</v>
+      </c>
+      <c r="F3" s="0">
+        <v>0.120461355894804</v>
+      </c>
+      <c r="G3" s="0">
+        <v>1527.4349670410156</v>
+      </c>
+      <c r="H3" s="0">
+        <v>24.999059200286865</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="B4" s="0" t="s">
         <v>5</v>
       </c>
       <c r="C4" s="0">
-        <v>50.863615984466769</v>
+        <v>69.993677139282227</v>
       </c>
       <c r="D4" s="0">
-        <v>4.0615902432434581</v>
+        <v>5.9923050403594971</v>
       </c>
       <c r="E4" s="0">
-        <v>17.344805500903654</v>
+        <v>1.9971457719802857</v>
+      </c>
+      <c r="F4" s="0">
+        <v>0.19971457496285439</v>
+      </c>
+      <c r="G4" s="0">
+        <v>3000.7096557617188</v>
+      </c>
+      <c r="H4" s="0">
+        <v>25.108068466186524</v>
       </c>
     </row>
     <row r="5">
@@ -218,6 +272,57 @@
         <v>17.344805500903654</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="C8" s="0">
+        <v>29.951983451843262</v>
+      </c>
+      <c r="D8" s="0">
+        <v>2.0092977285385132</v>
+      </c>
+      <c r="E8" s="0">
+        <v>0.4996095597743988</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9" s="0">
+        <v>50.012110710144043</v>
+      </c>
+      <c r="D9" s="0">
+        <v>4.0067151188850403</v>
+      </c>
+      <c r="E9" s="0">
+        <v>1.1990136802196503</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="B10" s="0" t="s">
+        <v>5</v>
+      </c>
+      <c r="C10" s="0">
+        <v>69.961456298828125</v>
+      </c>
+      <c r="D10" s="0">
+        <v>6.013290286064148</v>
+      </c>
+      <c r="E10" s="0">
+        <v>1.9959091246128082</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>